<commit_message>
Record 35 township education sessions for 3-1/3-2
Adds the nine townships' education reports (35 sessions, 7.8.-8.28.)
and replaces the earlier per-township estimate with one row per session:
target group, date, attendance, place. Each session ran one hour per the
county, for 36.5 hours with the budget school. The reports themselves
show no duration, so the sheet flags that the evidence needs it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YMTPih3wY83MLhP8gBywJV
</commit_message>
<xml_diff>
--- a/docs/취합서식/2026 성과평가 자료 취합 서식(1-1, 1-6, 3-1·3-2).xlsx
+++ b/docs/취합서식/2026 성과평가 자료 취합 서식(1-1, 1-6, 3-1·3-2).xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1714" uniqueCount="560">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1896" uniqueCount="605">
   <si>
     <r>
       <rPr>
@@ -22731,925 +22731,229 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주민참여예산 지역회의 교육</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">옥천읍</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">이장협의회</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(옥천읍 마을이장)</t>
   </si>
   <si>
     <t xml:space="preserve">옥천군(옥천읍)</t>
   </si>
   <si>
-    <t xml:space="preserve">주민참여예산제도 설명</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">옥천읍 지역회의 교육 결과보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제출 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">시간</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">×4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">회</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일자</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">인원 확인 필요</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주민참여예산 지역회의 교육</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">동이면</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">옥천군 주민참여예산 운영개요, 지역회의 역할 및 참여방법, 옥천군 주요 재정 현황</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(옥천읍) / 옥천읍행정복지센터 소회의실 / 11:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1시간(담당자 확인). 증빙에 종료시각·소요시간 기재 필요</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민자치회</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(옥천읍 주민자치위원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(옥천읍) / 옥천읍행정복지센터 소회의실 / 18:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">새마을단체</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(옥천읍 새마을지도자)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(옥천읍) / 옥천읍행정복지센터 소회의실 / 10:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">체육회</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(옥천읍 체육회원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(옥천읍) / 옥천읍행정복지센터 소회의실 / 18:30 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(동이면 주민자치회)</t>
   </si>
   <si>
     <t xml:space="preserve">옥천군(동이면)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">동이면 지역회의 교육 결과보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제출 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주민참여예산 지역회의 교육</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">안남면</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(동이면) / 다목적회관 2층 회의실</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(동이면 이장협의회)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기관단체협의회</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(동이면 기관단체협의회)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(동이면 새마을협의회)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기간제근로자</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(안남면 기간제근로자)</t>
   </si>
   <si>
     <t xml:space="preserve">옥천군(안남면)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">안남면 지역회의 교육 결과보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제출 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주민참여예산 지역회의 교육</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">안내면</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(안남면) / 안남면사무소 대회의실</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(안남면 이장협의회)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(안남면 주민자치회)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(안남면) / 안남면 다목적회관</t>
+  </si>
+  <si>
+    <t xml:space="preserve">지역사회보장협의체</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(안남면 지역사회보장협의체)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(안내면 주민자치회 위원)</t>
   </si>
   <si>
     <t xml:space="preserve">옥천군(안내면)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">안내면 지역회의 교육 결과보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제출 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주민참여예산 지역회의 교육</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">청성면</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(안내면) / 안내면행정복지센터 대회의실 / 9:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(안내면 이장)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(안내면) / 안내면행정복지센터 대회의실 / 10:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(안내면 새마을협의회)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(안내면) / 안내면행정복지센터 대회의실 / 14:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(안내면 기관단체장)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(안내면) / 면장실 / 11:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(청성면 마을이장)</t>
   </si>
   <si>
     <t xml:space="preserve">옥천군(청성면)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">청성면 지역회의 교육 결과보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제출 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주민참여예산 지역회의 교육</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">청산면</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(청성면) / 청성면행정복지센터 대회의실 / 10:50 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(청성면 새마을지도자)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(청성면) / 청성면행정복지센터 대회의실 / 11:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(청성면 주민자치위원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(청성면) / 청성면다목적회관 대회의실 / 15:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(청성면 기관단체장)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(청산면 주민자치회원)</t>
   </si>
   <si>
     <t xml:space="preserve">옥천군(청산면)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">청산면 지역회의 교육 결과보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제출 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주민참여예산 지역회의 교육</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이원면</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(청산면) / 청산면 다목적회관 2층 / 14:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(청산면 이장단)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(청산면) / 청산면 행정복지센터 다목적실 / 10:30 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">어르신 명예경찰</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(청산면 어르신 명예경찰)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(청산면) / 청산면 행정복지센터 다목적실 / 11:00 시작</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(청산면 새마을지도자회)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(이원면 주민자치위원)</t>
   </si>
   <si>
     <t xml:space="preserve">옥천군(이원면)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이원면 지역회의 교육 결과보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제출 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주민참여예산 지역회의 교육</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">군서면</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(이원면) / 면사무소 대회의실</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(이원면 이장)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(군서면 주민자치위원)</t>
   </si>
   <si>
     <t xml:space="preserve">옥천군(군서면)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">군서면 지역회의 교육 결과보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제출 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">2026 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">주민참여예산 지역회의 교육</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">군북면</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(군서면) / 군서면 대회의실</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(군서면 기관단체회의)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(군서면 새마을회)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(군서면 이장협의회)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(군북면 주민자치위원)</t>
   </si>
   <si>
     <t xml:space="preserve">옥천군(군북면)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">군북면 지역회의 교육 결과보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제출 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">■ 집계 (예시 행 제외)</t>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(군북면) / 군북면다목적회관 대회의실</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(군북면 지역사회보장협의회 위원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육실적(군북면) / 군북면사무소 회의실</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(군북면 기관단체기업체협의회 위원)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주민참여예산 홍보 및 교육(군북면 이장)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">■ 집계</t>
   </si>
   <si>
     <t xml:space="preserve">교육과정 수(교육대상 종류)</t>
@@ -23659,10 +22963,9 @@
       <rPr>
         <b val="true"/>
         <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3-1 </t>
     </r>
@@ -23670,7 +22973,6 @@
       <rPr>
         <b val="true"/>
         <sz val="10"/>
-        <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -23685,10 +22987,9 @@
       <rPr>
         <b val="true"/>
         <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="맑은 고딕"/>
-        <family val="3"/>
-        <charset val="129"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
       <t xml:space="preserve">3-2 </t>
     </r>
@@ -23696,7 +22997,6 @@
       <rPr>
         <b val="true"/>
         <sz val="10"/>
-        <color rgb="FF000000"/>
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
@@ -23704,7 +23004,7 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">※ 같은 대상에 같은 과정을 여러 번 운영했으면 과정 수는 1개로 보고, 시간은 모두 더해요.</t>
+    <t xml:space="preserve">※ 읍면 교육 35회(회당 1시간, 담당자 확인)는 대상만 다르고 내용이 같아요. 대상별로 세면 과정 수가 5개를 넘지만, 평가위원이 1과정으로 볼 수도 있어요(보수적으로는 예산학교 포함 2과정). 증빙 서식에 교육시간이 없으니 읍면 증빙에 시간을 보완하세요.</t>
   </si>
 </sst>
 </file>
@@ -23720,7 +23020,7 @@
     <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -23866,6 +23166,39 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -23942,7 +23275,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -24063,15 +23396,19 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="4" borderId="1" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="23" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -32603,7 +31940,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K48"/>
   <sheetFormatPr defaultColWidth="8.71484375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -32739,30 +32076,34 @@
         <v>2</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="C7" s="16" t="s">
         <v>525</v>
       </c>
-      <c r="D7" s="23"/>
+      <c r="C7" s="17" t="s">
+        <v>526</v>
+      </c>
+      <c r="D7" s="23" t="n">
+        <v>46211</v>
+      </c>
       <c r="E7" s="29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>521</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>526</v>
-      </c>
-      <c r="H7" s="16"/>
-      <c r="I7" s="30" t="s">
         <v>527</v>
       </c>
-      <c r="J7" s="30" t="s">
+      <c r="H7" s="16" t="n">
+        <v>61</v>
+      </c>
+      <c r="I7" s="17" t="s">
         <v>528</v>
       </c>
-      <c r="K7" s="16" t="s">
+      <c r="J7" s="17" t="s">
         <v>529</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32771,30 +32112,34 @@
         <v>3</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="C8" s="16" t="s">
-        <v>530</v>
-      </c>
-      <c r="D8" s="23"/>
+        <v>531</v>
+      </c>
+      <c r="C8" s="17" t="s">
+        <v>532</v>
+      </c>
+      <c r="D8" s="23" t="n">
+        <v>46217</v>
+      </c>
       <c r="E8" s="29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F8" s="17" t="s">
         <v>521</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>531</v>
-      </c>
-      <c r="H8" s="16"/>
-      <c r="I8" s="30" t="s">
         <v>527</v>
       </c>
-      <c r="J8" s="30" t="s">
-        <v>532</v>
-      </c>
-      <c r="K8" s="16" t="s">
-        <v>529</v>
+      <c r="H8" s="16" t="n">
+        <v>45</v>
+      </c>
+      <c r="I8" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J8" s="17" t="s">
+        <v>533</v>
+      </c>
+      <c r="K8" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32803,30 +32148,34 @@
         <v>4</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>533</v>
-      </c>
-      <c r="D9" s="23"/>
+        <v>534</v>
+      </c>
+      <c r="C9" s="17" t="s">
+        <v>535</v>
+      </c>
+      <c r="D9" s="23" t="n">
+        <v>46223</v>
+      </c>
       <c r="E9" s="29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F9" s="17" t="s">
         <v>521</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>534</v>
-      </c>
-      <c r="H9" s="16"/>
-      <c r="I9" s="30" t="s">
         <v>527</v>
       </c>
-      <c r="J9" s="30" t="s">
-        <v>535</v>
-      </c>
-      <c r="K9" s="16" t="s">
-        <v>529</v>
+      <c r="H9" s="16" t="n">
+        <v>60</v>
+      </c>
+      <c r="I9" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J9" s="17" t="s">
+        <v>536</v>
+      </c>
+      <c r="K9" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32835,30 +32184,34 @@
         <v>5</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="C10" s="16" t="s">
-        <v>536</v>
-      </c>
-      <c r="D10" s="23"/>
+        <v>537</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>538</v>
+      </c>
+      <c r="D10" s="23" t="n">
+        <v>46225</v>
+      </c>
       <c r="E10" s="29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F10" s="17" t="s">
         <v>521</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>537</v>
-      </c>
-      <c r="H10" s="16"/>
-      <c r="I10" s="30" t="s">
         <v>527</v>
       </c>
-      <c r="J10" s="30" t="s">
-        <v>538</v>
-      </c>
-      <c r="K10" s="16" t="s">
-        <v>529</v>
+      <c r="H10" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="I10" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J10" s="17" t="s">
+        <v>539</v>
+      </c>
+      <c r="K10" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32867,30 +32220,34 @@
         <v>6</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="C11" s="16" t="s">
-        <v>539</v>
-      </c>
-      <c r="D11" s="23"/>
+        <v>531</v>
+      </c>
+      <c r="C11" s="17" t="s">
+        <v>540</v>
+      </c>
+      <c r="D11" s="23" t="n">
+        <v>46211</v>
+      </c>
       <c r="E11" s="29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F11" s="17" t="s">
         <v>521</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>540</v>
-      </c>
-      <c r="H11" s="16"/>
-      <c r="I11" s="30" t="s">
-        <v>527</v>
-      </c>
-      <c r="J11" s="30" t="s">
         <v>541</v>
       </c>
-      <c r="K11" s="16" t="s">
-        <v>529</v>
+      <c r="H11" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="I11" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J11" s="17" t="s">
+        <v>542</v>
+      </c>
+      <c r="K11" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32899,30 +32256,34 @@
         <v>7</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="C12" s="16" t="s">
-        <v>542</v>
-      </c>
-      <c r="D12" s="23"/>
+        <v>525</v>
+      </c>
+      <c r="C12" s="17" t="s">
+        <v>543</v>
+      </c>
+      <c r="D12" s="23" t="n">
+        <v>46212</v>
+      </c>
       <c r="E12" s="29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F12" s="17" t="s">
         <v>521</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>543</v>
-      </c>
-      <c r="H12" s="16"/>
-      <c r="I12" s="30" t="s">
-        <v>527</v>
-      </c>
-      <c r="J12" s="30" t="s">
-        <v>544</v>
-      </c>
-      <c r="K12" s="16" t="s">
-        <v>529</v>
+        <v>541</v>
+      </c>
+      <c r="H12" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="I12" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J12" s="17" t="s">
+        <v>542</v>
+      </c>
+      <c r="K12" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32931,30 +32292,34 @@
         <v>8</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="C13" s="16" t="s">
+        <v>544</v>
+      </c>
+      <c r="C13" s="17" t="s">
         <v>545</v>
       </c>
-      <c r="D13" s="23"/>
+      <c r="D13" s="23" t="n">
+        <v>46213</v>
+      </c>
       <c r="E13" s="29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>521</v>
       </c>
       <c r="G13" s="17" t="s">
-        <v>546</v>
-      </c>
-      <c r="H13" s="16"/>
-      <c r="I13" s="30" t="s">
-        <v>527</v>
-      </c>
-      <c r="J13" s="30" t="s">
-        <v>547</v>
-      </c>
-      <c r="K13" s="16" t="s">
-        <v>529</v>
+        <v>541</v>
+      </c>
+      <c r="H13" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="I13" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J13" s="17" t="s">
+        <v>542</v>
+      </c>
+      <c r="K13" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32963,30 +32328,34 @@
         <v>9</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>548</v>
-      </c>
-      <c r="D14" s="23"/>
+        <v>534</v>
+      </c>
+      <c r="C14" s="17" t="s">
+        <v>546</v>
+      </c>
+      <c r="D14" s="23" t="n">
+        <v>46219</v>
+      </c>
       <c r="E14" s="29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>521</v>
       </c>
       <c r="G14" s="17" t="s">
-        <v>549</v>
-      </c>
-      <c r="H14" s="16"/>
-      <c r="I14" s="30" t="s">
-        <v>527</v>
-      </c>
-      <c r="J14" s="30" t="s">
-        <v>550</v>
-      </c>
-      <c r="K14" s="16" t="s">
-        <v>529</v>
+        <v>541</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <v>38</v>
+      </c>
+      <c r="I14" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J14" s="17" t="s">
+        <v>542</v>
+      </c>
+      <c r="K14" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -32995,316 +32364,1016 @@
         <v>10</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>486</v>
-      </c>
-      <c r="C15" s="16" t="s">
-        <v>551</v>
-      </c>
-      <c r="D15" s="23"/>
+        <v>547</v>
+      </c>
+      <c r="C15" s="17" t="s">
+        <v>548</v>
+      </c>
+      <c r="D15" s="23" t="n">
+        <v>46227</v>
+      </c>
       <c r="E15" s="29" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="F15" s="17" t="s">
         <v>521</v>
       </c>
       <c r="G15" s="17" t="s">
-        <v>552</v>
-      </c>
-      <c r="H15" s="16"/>
-      <c r="I15" s="30" t="s">
-        <v>527</v>
-      </c>
-      <c r="J15" s="30" t="s">
-        <v>553</v>
-      </c>
-      <c r="K15" s="16" t="s">
-        <v>529</v>
+        <v>549</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="I15" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J15" s="17" t="s">
+        <v>550</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="str">
+      <c r="A16" s="15" t="n">
         <f aca="false">IF(C16="","",COUNTA(C$6:C16))</f>
-        <v/>
-      </c>
-      <c r="B16" s="17"/>
-      <c r="C16" s="16"/>
-      <c r="D16" s="23"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="17"/>
-      <c r="G16" s="17"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="16"/>
-      <c r="J16" s="16"/>
-      <c r="K16" s="16"/>
+        <v>11</v>
+      </c>
+      <c r="B16" s="17" t="s">
+        <v>525</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>551</v>
+      </c>
+      <c r="D16" s="23" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E16" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G16" s="17" t="s">
+        <v>549</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="I16" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J16" s="17" t="s">
+        <v>550</v>
+      </c>
+      <c r="K16" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="15" t="str">
+      <c r="A17" s="15" t="n">
         <f aca="false">IF(C17="","",COUNTA(C$6:C17))</f>
-        <v/>
-      </c>
-      <c r="B17" s="17"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="29"/>
-      <c r="F17" s="17"/>
-      <c r="G17" s="17"/>
-      <c r="H17" s="16"/>
-      <c r="I17" s="16"/>
-      <c r="J17" s="16"/>
-      <c r="K17" s="16"/>
+        <v>12</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>552</v>
+      </c>
+      <c r="D17" s="23" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E17" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G17" s="17" t="s">
+        <v>549</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>31</v>
+      </c>
+      <c r="I17" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J17" s="17" t="s">
+        <v>553</v>
+      </c>
+      <c r="K17" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="15" t="str">
+      <c r="A18" s="15" t="n">
         <f aca="false">IF(C18="","",COUNTA(C$6:C18))</f>
-        <v/>
-      </c>
-      <c r="B18" s="17"/>
-      <c r="C18" s="16"/>
-      <c r="D18" s="23"/>
-      <c r="E18" s="29"/>
-      <c r="F18" s="17"/>
-      <c r="G18" s="17"/>
-      <c r="H18" s="16"/>
-      <c r="I18" s="16"/>
-      <c r="J18" s="16"/>
-      <c r="K18" s="16"/>
+        <v>13</v>
+      </c>
+      <c r="B18" s="17" t="s">
+        <v>554</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>555</v>
+      </c>
+      <c r="D18" s="23" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E18" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G18" s="17" t="s">
+        <v>549</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="I18" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J18" s="17" t="s">
+        <v>550</v>
+      </c>
+      <c r="K18" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="15" t="str">
+      <c r="A19" s="15" t="n">
         <f aca="false">IF(C19="","",COUNTA(C$6:C19))</f>
-        <v/>
-      </c>
-      <c r="B19" s="17"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="29"/>
-      <c r="F19" s="17"/>
-      <c r="G19" s="17"/>
-      <c r="H19" s="16"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="16"/>
-      <c r="K19" s="16"/>
+        <v>14</v>
+      </c>
+      <c r="B19" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="C19" s="17" t="s">
+        <v>556</v>
+      </c>
+      <c r="D19" s="23" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E19" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G19" s="17" t="s">
+        <v>557</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="I19" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J19" s="17" t="s">
+        <v>558</v>
+      </c>
+      <c r="K19" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="str">
+      <c r="A20" s="15" t="n">
         <f aca="false">IF(C20="","",COUNTA(C$6:C20))</f>
-        <v/>
-      </c>
-      <c r="B20" s="17"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="23"/>
-      <c r="E20" s="29"/>
-      <c r="F20" s="17"/>
-      <c r="G20" s="17"/>
-      <c r="H20" s="16"/>
-      <c r="I20" s="16"/>
-      <c r="J20" s="16"/>
-      <c r="K20" s="16"/>
+        <v>15</v>
+      </c>
+      <c r="B20" s="17" t="s">
+        <v>525</v>
+      </c>
+      <c r="C20" s="17" t="s">
+        <v>559</v>
+      </c>
+      <c r="D20" s="23" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E20" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G20" s="17" t="s">
+        <v>557</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="I20" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J20" s="17" t="s">
+        <v>560</v>
+      </c>
+      <c r="K20" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="15" t="str">
+      <c r="A21" s="15" t="n">
         <f aca="false">IF(C21="","",COUNTA(C$6:C21))</f>
-        <v/>
-      </c>
-      <c r="B21" s="17"/>
-      <c r="C21" s="16"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="29"/>
-      <c r="F21" s="17"/>
-      <c r="G21" s="17"/>
-      <c r="H21" s="16"/>
-      <c r="I21" s="16"/>
-      <c r="J21" s="16"/>
-      <c r="K21" s="16"/>
+        <v>16</v>
+      </c>
+      <c r="B21" s="17" t="s">
+        <v>534</v>
+      </c>
+      <c r="C21" s="17" t="s">
+        <v>561</v>
+      </c>
+      <c r="D21" s="23" t="n">
+        <v>46245</v>
+      </c>
+      <c r="E21" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G21" s="17" t="s">
+        <v>557</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="I21" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J21" s="17" t="s">
+        <v>562</v>
+      </c>
+      <c r="K21" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="15" t="str">
+      <c r="A22" s="15" t="n">
         <f aca="false">IF(C22="","",COUNTA(C$6:C22))</f>
-        <v/>
-      </c>
-      <c r="B22" s="17"/>
-      <c r="C22" s="16"/>
-      <c r="D22" s="23"/>
-      <c r="E22" s="29"/>
-      <c r="F22" s="17"/>
-      <c r="G22" s="17"/>
-      <c r="H22" s="16"/>
-      <c r="I22" s="16"/>
-      <c r="J22" s="16"/>
-      <c r="K22" s="16"/>
+        <v>17</v>
+      </c>
+      <c r="B22" s="17" t="s">
+        <v>544</v>
+      </c>
+      <c r="C22" s="17" t="s">
+        <v>563</v>
+      </c>
+      <c r="D22" s="23" t="n">
+        <v>46259</v>
+      </c>
+      <c r="E22" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G22" s="17" t="s">
+        <v>557</v>
+      </c>
+      <c r="H22" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="I22" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J22" s="17" t="s">
+        <v>564</v>
+      </c>
+      <c r="K22" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="15" t="str">
+      <c r="A23" s="15" t="n">
         <f aca="false">IF(C23="","",COUNTA(C$6:C23))</f>
-        <v/>
-      </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="23"/>
-      <c r="E23" s="29"/>
-      <c r="F23" s="17"/>
-      <c r="G23" s="17"/>
-      <c r="H23" s="16"/>
-      <c r="I23" s="16"/>
-      <c r="J23" s="16"/>
-      <c r="K23" s="16"/>
+        <v>18</v>
+      </c>
+      <c r="B23" s="17" t="s">
+        <v>525</v>
+      </c>
+      <c r="C23" s="17" t="s">
+        <v>565</v>
+      </c>
+      <c r="D23" s="23" t="n">
+        <v>46238</v>
+      </c>
+      <c r="E23" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G23" s="17" t="s">
+        <v>566</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="I23" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J23" s="17" t="s">
+        <v>567</v>
+      </c>
+      <c r="K23" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="15" t="str">
+      <c r="A24" s="15" t="n">
         <f aca="false">IF(C24="","",COUNTA(C$6:C24))</f>
-        <v/>
-      </c>
-      <c r="B24" s="17"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="23"/>
-      <c r="E24" s="29"/>
-      <c r="F24" s="17"/>
-      <c r="G24" s="17"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
-      <c r="J24" s="16"/>
-      <c r="K24" s="16"/>
+        <v>19</v>
+      </c>
+      <c r="B24" s="17" t="s">
+        <v>534</v>
+      </c>
+      <c r="C24" s="17" t="s">
+        <v>568</v>
+      </c>
+      <c r="D24" s="23" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E24" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G24" s="17" t="s">
+        <v>566</v>
+      </c>
+      <c r="H24" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="I24" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J24" s="17" t="s">
+        <v>569</v>
+      </c>
+      <c r="K24" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="15" t="str">
+      <c r="A25" s="15" t="n">
         <f aca="false">IF(C25="","",COUNTA(C$6:C25))</f>
-        <v/>
-      </c>
-      <c r="B25" s="17"/>
-      <c r="C25" s="16"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="29"/>
-      <c r="F25" s="17"/>
-      <c r="G25" s="17"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
-      <c r="J25" s="16"/>
-      <c r="K25" s="16"/>
+        <v>20</v>
+      </c>
+      <c r="B25" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="C25" s="17" t="s">
+        <v>570</v>
+      </c>
+      <c r="D25" s="23" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E25" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G25" s="17" t="s">
+        <v>566</v>
+      </c>
+      <c r="H25" s="16" t="n">
+        <v>35</v>
+      </c>
+      <c r="I25" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J25" s="17" t="s">
+        <v>571</v>
+      </c>
+      <c r="K25" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="15" t="str">
+      <c r="A26" s="15" t="n">
         <f aca="false">IF(C26="","",COUNTA(C$6:C26))</f>
-        <v/>
-      </c>
-      <c r="B26" s="17"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="23"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="17"/>
-      <c r="G26" s="17"/>
-      <c r="H26" s="16"/>
-      <c r="I26" s="16"/>
-      <c r="J26" s="16"/>
-      <c r="K26" s="16"/>
+        <v>21</v>
+      </c>
+      <c r="B26" s="17" t="s">
+        <v>544</v>
+      </c>
+      <c r="C26" s="17" t="s">
+        <v>572</v>
+      </c>
+      <c r="D26" s="23" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E26" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G26" s="17" t="s">
+        <v>566</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="I26" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J26" s="17" t="s">
+        <v>569</v>
+      </c>
+      <c r="K26" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="15" t="str">
+      <c r="A27" s="15" t="n">
         <f aca="false">IF(C27="","",COUNTA(C$6:C27))</f>
-        <v/>
-      </c>
-      <c r="B27" s="17"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="23"/>
-      <c r="E27" s="29"/>
-      <c r="F27" s="17"/>
-      <c r="G27" s="17"/>
-      <c r="H27" s="16"/>
-      <c r="I27" s="16"/>
-      <c r="J27" s="16"/>
-      <c r="K27" s="16"/>
+        <v>22</v>
+      </c>
+      <c r="B27" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>573</v>
+      </c>
+      <c r="D27" s="23" t="n">
+        <v>46230</v>
+      </c>
+      <c r="E27" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G27" s="17" t="s">
+        <v>574</v>
+      </c>
+      <c r="H27" s="16" t="n">
+        <v>28</v>
+      </c>
+      <c r="I27" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J27" s="17" t="s">
+        <v>575</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="15" t="str">
+      <c r="A28" s="15" t="n">
         <f aca="false">IF(C28="","",COUNTA(C$6:C28))</f>
-        <v/>
-      </c>
-      <c r="B28" s="17"/>
-      <c r="C28" s="16"/>
-      <c r="D28" s="23"/>
-      <c r="E28" s="29"/>
-      <c r="F28" s="17"/>
-      <c r="G28" s="17"/>
-      <c r="H28" s="16"/>
-      <c r="I28" s="16"/>
-      <c r="J28" s="16"/>
-      <c r="K28" s="16"/>
+        <v>23</v>
+      </c>
+      <c r="B28" s="17" t="s">
+        <v>525</v>
+      </c>
+      <c r="C28" s="17" t="s">
+        <v>576</v>
+      </c>
+      <c r="D28" s="23" t="n">
+        <v>46240</v>
+      </c>
+      <c r="E28" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G28" s="17" t="s">
+        <v>574</v>
+      </c>
+      <c r="H28" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="I28" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J28" s="17" t="s">
+        <v>577</v>
+      </c>
+      <c r="K28" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="15" t="str">
+      <c r="A29" s="15" t="n">
         <f aca="false">IF(C29="","",COUNTA(C$6:C29))</f>
-        <v/>
-      </c>
-      <c r="B29" s="17"/>
-      <c r="C29" s="16"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="29"/>
-      <c r="F29" s="17"/>
-      <c r="G29" s="17"/>
-      <c r="H29" s="16"/>
-      <c r="I29" s="16"/>
-      <c r="J29" s="16"/>
-      <c r="K29" s="16"/>
+        <v>24</v>
+      </c>
+      <c r="B29" s="17" t="s">
+        <v>578</v>
+      </c>
+      <c r="C29" s="17" t="s">
+        <v>579</v>
+      </c>
+      <c r="D29" s="23" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E29" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G29" s="17" t="s">
+        <v>574</v>
+      </c>
+      <c r="H29" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="I29" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J29" s="17" t="s">
+        <v>580</v>
+      </c>
+      <c r="K29" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="15" t="str">
+      <c r="A30" s="15" t="n">
         <f aca="false">IF(C30="","",COUNTA(C$6:C30))</f>
-        <v/>
-      </c>
-      <c r="B30" s="17"/>
-      <c r="C30" s="16"/>
-      <c r="D30" s="23"/>
-      <c r="E30" s="29"/>
-      <c r="F30" s="17"/>
-      <c r="G30" s="17"/>
-      <c r="H30" s="16"/>
-      <c r="I30" s="16"/>
-      <c r="J30" s="16"/>
-      <c r="K30" s="16"/>
+        <v>25</v>
+      </c>
+      <c r="B30" s="17" t="s">
+        <v>534</v>
+      </c>
+      <c r="C30" s="17" t="s">
+        <v>581</v>
+      </c>
+      <c r="D30" s="23" t="n">
+        <v>46248</v>
+      </c>
+      <c r="E30" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G30" s="17" t="s">
+        <v>574</v>
+      </c>
+      <c r="H30" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="I30" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J30" s="17" t="s">
+        <v>580</v>
+      </c>
+      <c r="K30" s="17" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15" t="n">
+        <f aca="false">IF(C31="","",COUNTA(C$6:C31))</f>
+        <v>26</v>
+      </c>
+      <c r="B31" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="C31" s="17" t="s">
+        <v>582</v>
+      </c>
+      <c r="D31" s="23" t="n">
+        <v>46216</v>
+      </c>
+      <c r="E31" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G31" s="17" t="s">
+        <v>583</v>
+      </c>
+      <c r="H31" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="I31" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J31" s="17" t="s">
+        <v>584</v>
+      </c>
+      <c r="K31" s="17" t="s">
+        <v>530</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="13" t="s">
-        <v>554</v>
+      <c r="A32" s="15" t="n">
+        <f aca="false">IF(C32="","",COUNTA(C$6:C32))</f>
+        <v>27</v>
+      </c>
+      <c r="B32" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="C32" s="17" t="s">
+        <v>582</v>
+      </c>
+      <c r="D32" s="23" t="n">
+        <v>46244</v>
+      </c>
+      <c r="E32" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G32" s="17" t="s">
+        <v>583</v>
+      </c>
+      <c r="H32" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="I32" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J32" s="17" t="s">
+        <v>584</v>
+      </c>
+      <c r="K32" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="24" t="s">
-        <v>555</v>
-      </c>
-      <c r="C33" s="31" t="n">
-        <f aca="false">SUMPRODUCT((B6:B30&lt;&gt;"")/COUNTIF(B6:B30,B6:B30&amp;""))</f>
-        <v>2</v>
+      <c r="A33" s="15" t="n">
+        <f aca="false">IF(C33="","",COUNTA(C$6:C33))</f>
+        <v>28</v>
+      </c>
+      <c r="B33" s="17" t="s">
+        <v>525</v>
+      </c>
+      <c r="C33" s="17" t="s">
+        <v>585</v>
+      </c>
+      <c r="D33" s="23" t="n">
+        <v>46253</v>
+      </c>
+      <c r="E33" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G33" s="17" t="s">
+        <v>583</v>
+      </c>
+      <c r="H33" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="I33" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J33" s="17" t="s">
+        <v>584</v>
+      </c>
+      <c r="K33" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="32" t="s">
-        <v>556</v>
-      </c>
-      <c r="C34" s="31" t="n">
-        <f aca="false">IF(C33&gt;=5,4,IF(C33&gt;=3,3,IF(C33&gt;=1,2,0)))</f>
-        <v>2</v>
+      <c r="A34" s="15" t="n">
+        <f aca="false">IF(C34="","",COUNTA(C$6:C34))</f>
+        <v>29</v>
+      </c>
+      <c r="B34" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="C34" s="17" t="s">
+        <v>586</v>
+      </c>
+      <c r="D34" s="23" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E34" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G34" s="17" t="s">
+        <v>587</v>
+      </c>
+      <c r="H34" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="I34" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J34" s="17" t="s">
+        <v>588</v>
+      </c>
+      <c r="K34" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="24" t="s">
-        <v>557</v>
-      </c>
-      <c r="C35" s="31" t="n">
-        <f aca="false">SUM(E6:E30)</f>
-        <v>37.5</v>
+      <c r="A35" s="15" t="n">
+        <f aca="false">IF(C35="","",COUNTA(C$6:C35))</f>
+        <v>30</v>
+      </c>
+      <c r="B35" s="17" t="s">
+        <v>544</v>
+      </c>
+      <c r="C35" s="17" t="s">
+        <v>589</v>
+      </c>
+      <c r="D35" s="23" t="n">
+        <v>46246</v>
+      </c>
+      <c r="E35" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G35" s="17" t="s">
+        <v>587</v>
+      </c>
+      <c r="H35" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="I35" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J35" s="17" t="s">
+        <v>588</v>
+      </c>
+      <c r="K35" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="32" t="s">
-        <v>558</v>
-      </c>
-      <c r="C36" s="31" t="n">
-        <f aca="false">IF(C35&gt;=15,4,IF(C35&gt;=7,2,0))</f>
-        <v>4</v>
+      <c r="A36" s="15" t="n">
+        <f aca="false">IF(C36="","",COUNTA(C$6:C36))</f>
+        <v>31</v>
+      </c>
+      <c r="B36" s="17" t="s">
+        <v>534</v>
+      </c>
+      <c r="C36" s="17" t="s">
+        <v>590</v>
+      </c>
+      <c r="D36" s="23" t="n">
+        <v>46247</v>
+      </c>
+      <c r="E36" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G36" s="17" t="s">
+        <v>587</v>
+      </c>
+      <c r="H36" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="I36" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J36" s="17" t="s">
+        <v>588</v>
+      </c>
+      <c r="K36" s="17" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="33" t="s">
-        <v>559</v>
+      <c r="A37" s="15" t="n">
+        <f aca="false">IF(C37="","",COUNTA(C$6:C37))</f>
+        <v>32</v>
+      </c>
+      <c r="B37" s="17" t="s">
+        <v>525</v>
+      </c>
+      <c r="C37" s="17" t="s">
+        <v>591</v>
+      </c>
+      <c r="D37" s="23" t="n">
+        <v>46262</v>
+      </c>
+      <c r="E37" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G37" s="17" t="s">
+        <v>587</v>
+      </c>
+      <c r="H37" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="I37" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J37" s="17" t="s">
+        <v>588</v>
+      </c>
+      <c r="K37" s="17" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="15" t="n">
+        <f aca="false">IF(C38="","",COUNTA(C$6:C38))</f>
+        <v>33</v>
+      </c>
+      <c r="B38" s="17" t="s">
+        <v>531</v>
+      </c>
+      <c r="C38" s="17" t="s">
+        <v>592</v>
+      </c>
+      <c r="D38" s="23" t="n">
+        <v>46217</v>
+      </c>
+      <c r="E38" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G38" s="17" t="s">
+        <v>593</v>
+      </c>
+      <c r="H38" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="I38" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J38" s="17" t="s">
+        <v>594</v>
+      </c>
+      <c r="K38" s="17" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="15" t="n">
+        <f aca="false">IF(C39="","",COUNTA(C$6:C39))</f>
+        <v>34</v>
+      </c>
+      <c r="B39" s="17" t="s">
+        <v>554</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>595</v>
+      </c>
+      <c r="D39" s="23" t="n">
+        <v>46223</v>
+      </c>
+      <c r="E39" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G39" s="17" t="s">
+        <v>593</v>
+      </c>
+      <c r="H39" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="I39" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J39" s="17" t="s">
+        <v>596</v>
+      </c>
+      <c r="K39" s="17" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="15" t="n">
+        <f aca="false">IF(C40="","",COUNTA(C$6:C40))</f>
+        <v>35</v>
+      </c>
+      <c r="B40" s="17" t="s">
+        <v>544</v>
+      </c>
+      <c r="C40" s="17" t="s">
+        <v>597</v>
+      </c>
+      <c r="D40" s="23" t="n">
+        <v>46224</v>
+      </c>
+      <c r="E40" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G40" s="17" t="s">
+        <v>593</v>
+      </c>
+      <c r="H40" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="I40" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J40" s="17" t="s">
+        <v>596</v>
+      </c>
+      <c r="K40" s="17" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="15" t="n">
+        <f aca="false">IF(C41="","",COUNTA(C$6:C41))</f>
+        <v>36</v>
+      </c>
+      <c r="B41" s="17" t="s">
+        <v>525</v>
+      </c>
+      <c r="C41" s="17" t="s">
+        <v>598</v>
+      </c>
+      <c r="D41" s="23" t="n">
+        <v>46239</v>
+      </c>
+      <c r="E41" s="29" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="17" t="s">
+        <v>521</v>
+      </c>
+      <c r="G41" s="17" t="s">
+        <v>593</v>
+      </c>
+      <c r="H41" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="I41" s="17" t="s">
+        <v>528</v>
+      </c>
+      <c r="J41" s="17" t="s">
+        <v>596</v>
+      </c>
+      <c r="K41" s="17" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B43" s="30" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B44" s="31" t="s">
+        <v>600</v>
+      </c>
+      <c r="C44" s="32" t="n">
+        <f aca="false">SUMPRODUCT((B6:B41&lt;&gt;"")/COUNTIF(B6:B41,B6:B41&amp;""))</f>
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B45" s="33" t="s">
+        <v>601</v>
+      </c>
+      <c r="C45" s="32" t="n">
+        <f aca="false">IF(C44&gt;=5,4,IF(C44&gt;=3,3,IF(C44&gt;=1,2,0)))</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B46" s="31" t="s">
+        <v>602</v>
+      </c>
+      <c r="C46" s="32" t="n">
+        <f aca="false">SUM(E6:E41)</f>
+        <v>36.5</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B47" s="33" t="s">
+        <v>603</v>
+      </c>
+      <c r="C47" s="32" t="n">
+        <f aca="false">IF(C46&gt;=15,4,IF(C46&gt;=7,2,0))</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B48" s="34" t="s">
+        <v>604</v>
       </c>
     </row>
   </sheetData>
@@ -33314,15 +33383,15 @@
     <mergeCell ref="A3:K3"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B6:B30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="B6:B41" type="list">
       <formula1>"참여예산주민위원회,지역회의,주민자치회 등 주민기구,사회적약자,아동·청소년,청년,일반주민,기타"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F6:F30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F6:F41" type="list">
       <formula1>"대면,온라인,혼합"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G6:G30" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G6:G41" type="list">
       <formula1>"옥천군,충청북도,위탁기관,기타"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>